<commit_message>
updaing x axis on dilution plot
</commit_message>
<xml_diff>
--- a/chapter_7/reductions-lit/data/dilution_data_extra.xlsx
+++ b/chapter_7/reductions-lit/data/dilution_data_extra.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/chapter_7/reductions-lit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{A159C0DB-AC25-4DE9-8CEC-DA3CD6C5DB26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E8377A3-26DA-4C4B-9465-44A6D16A7E81}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="8_{A159C0DB-AC25-4DE9-8CEC-DA3CD6C5DB26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{753B993C-4716-4EFF-8DE0-11752B70EF3B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{122F0065-8602-49EC-B7E3-7261009AF15D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="84">
   <si>
     <t>Table 5</t>
   </si>
@@ -258,6 +258,36 @@
   </si>
   <si>
     <t>dil.dm</t>
+  </si>
+  <si>
+    <t>1:0.25</t>
+  </si>
+  <si>
+    <t>1:0.5</t>
+  </si>
+  <si>
+    <t>1:0.2</t>
+  </si>
+  <si>
+    <t>1:0.4</t>
+  </si>
+  <si>
+    <t>1:0.6</t>
+  </si>
+  <si>
+    <t>1:0.8</t>
+  </si>
+  <si>
+    <t>1:1.2</t>
+  </si>
+  <si>
+    <t>1:1.4</t>
+  </si>
+  <si>
+    <t>1:1.5</t>
+  </si>
+  <si>
+    <t>1:2</t>
   </si>
 </sst>
 </file>
@@ -760,6 +790,9 @@
       <c r="H2" s="4">
         <v>0.25</v>
       </c>
+      <c r="I2" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="J2" s="1">
         <f>G2*(1/(1+H2))</f>
         <v>3.1680000000000001</v>
@@ -809,6 +842,9 @@
       <c r="H3" s="4">
         <v>0.5</v>
       </c>
+      <c r="I3" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J3" s="1">
         <f t="shared" ref="J3:J39" si="0">G3*(1/(1+H3))</f>
         <v>1.6600000000000001</v>
@@ -1060,6 +1096,9 @@
       <c r="H8" s="4">
         <v>0.2</v>
       </c>
+      <c r="I8" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="J8" s="1">
         <f t="shared" si="0"/>
         <v>8.75</v>
@@ -1103,6 +1142,9 @@
       <c r="H9" s="4">
         <v>0.4</v>
       </c>
+      <c r="I9" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="J9" s="1">
         <f t="shared" si="0"/>
         <v>7.5</v>
@@ -1143,6 +1185,9 @@
       <c r="H10" s="4">
         <v>0.6</v>
       </c>
+      <c r="I10" s="3" t="s">
+        <v>78</v>
+      </c>
       <c r="J10" s="1">
         <f t="shared" si="0"/>
         <v>6.5625</v>
@@ -1183,6 +1228,9 @@
       <c r="H11" s="4">
         <v>0.8</v>
       </c>
+      <c r="I11" s="3" t="s">
+        <v>79</v>
+      </c>
       <c r="J11" s="1">
         <f t="shared" si="0"/>
         <v>5.8333333333333339</v>
@@ -1266,6 +1314,9 @@
       <c r="H13" s="4">
         <v>1.2</v>
       </c>
+      <c r="I13" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="J13" s="1">
         <f t="shared" si="0"/>
         <v>4.7727272727272725</v>
@@ -1306,6 +1357,9 @@
       <c r="H14" s="4">
         <v>1.4</v>
       </c>
+      <c r="I14" s="3" t="s">
+        <v>81</v>
+      </c>
       <c r="J14" s="1">
         <f t="shared" si="0"/>
         <v>4.375</v>
@@ -1343,6 +1397,9 @@
       <c r="H15" s="4">
         <v>0.5</v>
       </c>
+      <c r="I15" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J15" s="1">
         <f t="shared" si="0"/>
         <v>6.8666666666666671</v>
@@ -1442,6 +1499,9 @@
       <c r="H17" s="4">
         <v>1.5</v>
       </c>
+      <c r="I17" s="3" t="s">
+        <v>82</v>
+      </c>
       <c r="J17" s="1">
         <f t="shared" si="0"/>
         <v>4.12</v>
@@ -1490,6 +1550,9 @@
       <c r="H18" s="4">
         <v>0.5</v>
       </c>
+      <c r="I18" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J18" s="1">
         <f t="shared" si="0"/>
         <v>6.8666666666666671</v>
@@ -1589,6 +1652,9 @@
       <c r="H20" s="4">
         <v>1.5</v>
       </c>
+      <c r="I20" s="3" t="s">
+        <v>82</v>
+      </c>
       <c r="J20" s="1">
         <f t="shared" si="0"/>
         <v>4.12</v>
@@ -1637,6 +1703,9 @@
       <c r="H21" s="4">
         <v>0.5</v>
       </c>
+      <c r="I21" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J21" s="1">
         <f t="shared" si="0"/>
         <v>6.8666666666666671</v>
@@ -1736,6 +1805,9 @@
       <c r="H23" s="4">
         <v>1.5</v>
       </c>
+      <c r="I23" s="3" t="s">
+        <v>82</v>
+      </c>
       <c r="J23" s="1">
         <f t="shared" si="0"/>
         <v>4.12</v>
@@ -1784,6 +1856,9 @@
       <c r="H24" s="4">
         <v>0.5</v>
       </c>
+      <c r="I24" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J24" s="1">
         <f t="shared" si="0"/>
         <v>6.8666666666666671</v>
@@ -1883,6 +1958,9 @@
       <c r="H26" s="4">
         <v>1.5</v>
       </c>
+      <c r="I26" s="3" t="s">
+        <v>82</v>
+      </c>
       <c r="J26" s="1">
         <f t="shared" si="0"/>
         <v>4.12</v>
@@ -1928,6 +2006,9 @@
       <c r="H27" s="4">
         <v>0.5</v>
       </c>
+      <c r="I27" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J27" s="1">
         <f t="shared" si="0"/>
         <v>5.333333333333333</v>
@@ -2017,6 +2098,9 @@
       <c r="H29" s="4">
         <v>2</v>
       </c>
+      <c r="I29" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="J29" s="1">
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
@@ -2060,6 +2144,9 @@
       <c r="H30" s="4">
         <v>0.5</v>
       </c>
+      <c r="I30" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J30" s="1">
         <f t="shared" si="0"/>
         <v>5.333333333333333</v>
@@ -2149,6 +2236,9 @@
       <c r="H32" s="4">
         <v>2</v>
       </c>
+      <c r="I32" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="J32" s="1">
         <f t="shared" si="0"/>
         <v>2.6666666666666665</v>
@@ -2192,6 +2282,9 @@
       <c r="H33" s="4">
         <v>0.5</v>
       </c>
+      <c r="I33" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="J33" s="1">
         <f t="shared" si="0"/>
         <v>5.333333333333333</v>
@@ -2280,6 +2373,9 @@
       </c>
       <c r="H35" s="4">
         <v>2</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="J35" s="1">
         <f t="shared" si="0"/>

</xml_diff>